<commit_message>
fix: vehicle labels, color coding, marker persistence and route cleanup
</commit_message>
<xml_diff>
--- a/sample_data/layout excel para app.xlsx
+++ b/sample_data/layout excel para app.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ec5c3f241efecdab/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\54116\projects\app-traslado-personal\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{3156E44D-01BC-4452-AA55-B7489F52593C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDBE6B50-395B-49FC-8C81-E390719C62C7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CEDDE1-A506-4606-8DDE-8133B943875B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{89C59B45-3584-4542-9C15-833B50F23AF3}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="71">
   <si>
     <t>Menu</t>
   </si>
@@ -77,9 +77,6 @@
   </si>
   <si>
     <t>Hay una cocina de la casa (cuenta con 2 heladeras).</t>
-  </si>
-  <si>
-    <t>#######</t>
   </si>
   <si>
     <t>Profesion</t>
@@ -980,18 +977,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" t="s">
         <v>70</v>
-      </c>
-      <c r="B6" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>13</v>
+      <c r="B7" s="4">
+        <v>45884</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1040,48 +1037,48 @@
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="C1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="8" t="s">
         <v>20</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>21</v>
       </c>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>25</v>
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="12"/>
@@ -1090,20 +1087,20 @@
     </row>
     <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="14" t="s">
         <v>29</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>30</v>
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="16"/>
@@ -1112,20 +1109,20 @@
     </row>
     <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>34</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>35</v>
       </c>
       <c r="E4" s="11"/>
       <c r="F4" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="12"/>
@@ -1134,23 +1131,23 @@
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>39</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>40</v>
       </c>
       <c r="E5" s="15"/>
       <c r="F5" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" s="14" t="s">
         <v>41</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>42</v>
       </c>
       <c r="H5" s="16"/>
       <c r="I5" s="2"/>
@@ -1158,16 +1155,16 @@
     </row>
     <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="C6" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>46</v>
       </c>
       <c r="E6" s="10">
         <v>1754</v>
@@ -1180,20 +1177,20 @@
     </row>
     <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="14" t="s">
         <v>48</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>49</v>
       </c>
       <c r="E7" s="15"/>
       <c r="F7" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="16"/>
@@ -1202,23 +1199,23 @@
     </row>
     <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="D8" s="37" t="s">
         <v>52</v>
-      </c>
-      <c r="D8" s="37" t="s">
-        <v>53</v>
       </c>
       <c r="E8" s="40"/>
       <c r="F8" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="37" t="s">
         <v>54</v>
-      </c>
-      <c r="G8" s="37" t="s">
-        <v>55</v>
       </c>
       <c r="H8" s="29"/>
       <c r="I8" s="32"/>
@@ -1239,7 +1236,7 @@
     <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="36"/>
       <c r="B10" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C10" s="39"/>
       <c r="D10" s="39"/>
@@ -1252,13 +1249,13 @@
     </row>
     <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>56</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>57</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="15"/>
@@ -1296,13 +1293,13 @@
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="C1" s="22" t="s">
         <v>59</v>
-      </c>
-      <c r="C1" s="22" t="s">
-        <v>60</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -1314,7 +1311,7 @@
     </row>
     <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" s="24" t="s">
         <v>9</v>
@@ -1332,10 +1329,10 @@
     </row>
     <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="27" t="s">
         <v>61</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>62</v>
       </c>
       <c r="C3" s="28">
         <v>15</v>
@@ -1350,10 +1347,10 @@
     </row>
     <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="24" t="s">
         <v>63</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>64</v>
       </c>
       <c r="C4" s="25">
         <v>1</v>
@@ -1368,10 +1365,10 @@
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C5" s="28">
         <v>1</v>
@@ -1386,10 +1383,10 @@
     </row>
     <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="24" t="s">
         <v>66</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>67</v>
       </c>
       <c r="C6" s="25">
         <v>100</v>
@@ -1404,10 +1401,10 @@
     </row>
     <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C7" s="28">
         <v>15</v>
@@ -1422,10 +1419,10 @@
     </row>
     <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="24" t="s">
         <v>68</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>69</v>
       </c>
       <c r="C8" s="25">
         <v>108</v>

</xml_diff>